<commit_message>
Adicionado a geração de parametros de banco de dados e gravacao no SQLite
</commit_message>
<xml_diff>
--- a/Template Layout XLSX/Liberacoes.xlsx
+++ b/Template Layout XLSX/Liberacoes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcelo.rogoski\Documents\DMM\MigracaoDados\MigracaoDados\Template Layout XLSX\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CF5D6E4A-C2AC-4474-AA71-0716B883BCE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7674B9A9-BEE0-4CCA-9CA9-FD4E703119A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{338C9EAA-62CD-42AE-B7E5-9D583D79B191}"/>
+    <workbookView xWindow="-23130" yWindow="3000" windowWidth="21600" windowHeight="11235" xr2:uid="{338C9EAA-62CD-42AE-B7E5-9D583D79B191}"/>
   </bookViews>
   <sheets>
     <sheet name="Liberacoes" sheetId="1" r:id="rId1"/>
@@ -238,7 +238,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="55">
   <si>
     <t>ID</t>
   </si>
@@ -397,6 +397,12 @@
   </si>
   <si>
     <t>ENT_NR_CONTA</t>
+  </si>
+  <si>
+    <t>ENT_VL_MSOLIC</t>
+  </si>
+  <si>
+    <t>Valor M_Solicitado</t>
   </si>
 </sst>
 </file>
@@ -460,12 +466,18 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -496,7 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -524,6 +536,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -860,7 +884,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AFD48BD-0417-42D3-83A8-B7B5C3F766EC}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="4" customWidth="1"/>
@@ -1332,6 +1356,29 @@
       </c>
       <c r="G21" s="5"/>
     </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="10">
+        <v>20</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="12">
+        <v>17</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <headerFooter>

</xml_diff>